<commit_message>
Updated AUS_grids_kan50 model - 2026-09-06 21:23
</commit_message>
<xml_diff>
--- a/VerveStacks_AUS_grids_kan50/Sets-vervestacks.xlsx
+++ b/VerveStacks_AUS_grids_kan50/Sets-vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_AUS_grids_kan50\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4D043F3-49E7-4D5D-9234-6097430782D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{309B1715-43AF-412C-A9A2-5C32B97DB688}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1359" uniqueCount="735">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1371" uniqueCount="741">
   <si>
     <t>~TFM_Psets</t>
   </si>
@@ -584,6 +584,12 @@
     <t>*[_]Nebo_AUS</t>
   </si>
   <si>
+    <t>p_Dubbo_AUS</t>
+  </si>
+  <si>
+    <t>*[_]Dubbo_AUS</t>
+  </si>
+  <si>
     <t>p_MountPiper_AUS</t>
   </si>
   <si>
@@ -608,12 +614,6 @@
     <t>*[_]Tarong_AUS</t>
   </si>
   <si>
-    <t>p_Blackwall_AUS</t>
-  </si>
-  <si>
-    <t>*[_]Blackwall_AUS</t>
-  </si>
-  <si>
     <t>p_Bouldercombe_AUS</t>
   </si>
   <si>
@@ -644,6 +644,12 @@
     <t>*[_]Para_AUS</t>
   </si>
   <si>
+    <t>p_Brisbane_AUS</t>
+  </si>
+  <si>
+    <t>*[_]Brisbane_AUS</t>
+  </si>
+  <si>
     <t>p_BulliCreek_AUS</t>
   </si>
   <si>
@@ -728,6 +734,12 @@
     <t>*[_]AUS22p9S118p7E_AUS</t>
   </si>
   <si>
+    <t>p_Morawa_AUS</t>
+  </si>
+  <si>
+    <t>*[_]Morawa_AUS</t>
+  </si>
+  <si>
     <t>p_Canberra_AUS</t>
   </si>
   <si>
@@ -762,6 +774,12 @@
   </si>
   <si>
     <t>*[_]Horsham_AUS</t>
+  </si>
+  <si>
+    <t>p_PortHedland_AUS</t>
+  </si>
+  <si>
+    <t>*[_]PortHedland_AUS</t>
   </si>
   <si>
     <t>p_Kalgoorlie_AUS</t>
@@ -2996,7 +3014,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B9596CD-0528-4380-8F2D-D99C9A838BA1}">
-  <dimension ref="B9:E298"/>
+  <dimension ref="B9:E301"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
     <row r="9" spans="2:5" x14ac:dyDescent="0.45">
@@ -7047,6 +7065,48 @@
         <v>734</v>
       </c>
       <c r="E298" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="299" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B299" t="s">
+        <v>735</v>
+      </c>
+      <c r="C299" t="s">
+        <v>736</v>
+      </c>
+      <c r="D299" t="s">
+        <v>736</v>
+      </c>
+      <c r="E299" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="300" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B300" t="s">
+        <v>737</v>
+      </c>
+      <c r="C300" t="s">
+        <v>738</v>
+      </c>
+      <c r="D300" t="s">
+        <v>738</v>
+      </c>
+      <c r="E300" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="301" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B301" t="s">
+        <v>739</v>
+      </c>
+      <c r="C301" t="s">
+        <v>740</v>
+      </c>
+      <c r="D301" t="s">
+        <v>740</v>
+      </c>
+      <c r="E301" t="s">
         <v>149</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Updated AUS_grids_kan50 model - 2026-09-07 22:51
</commit_message>
<xml_diff>
--- a/VerveStacks_AUS_grids_kan50/Sets-vervestacks.xlsx
+++ b/VerveStacks_AUS_grids_kan50/Sets-vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_AUS_grids_kan50\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6176B94-9102-4B50-B283-CF0EA24E582A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF0F34DB-20C0-4CA3-8616-00863318CD1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1367" uniqueCount="739">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1375" uniqueCount="743">
   <si>
     <t>~TFM_Psets</t>
   </si>
@@ -662,6 +662,12 @@
     <t>*[_]Murray_AUS</t>
   </si>
   <si>
+    <t>p_OlympicDamWest_AUS</t>
+  </si>
+  <si>
+    <t>*[_]OlympicDamWest_AUS</t>
+  </si>
+  <si>
     <t>p_Chalumbin_AUS</t>
   </si>
   <si>
@@ -774,6 +780,12 @@
   </si>
   <si>
     <t>*[_]PortHedland_AUS</t>
+  </si>
+  <si>
+    <t>p_AUS42p8S146p2E_AUS</t>
+  </si>
+  <si>
+    <t>*[_]AUS42p8S146p2E_AUS</t>
   </si>
   <si>
     <t>p_Kalgoorlie_AUS</t>
@@ -3008,7 +3020,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B9596CD-0528-4380-8F2D-D99C9A838BA1}">
-  <dimension ref="B9:E300"/>
+  <dimension ref="B9:E302"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
     <row r="9" spans="2:5" x14ac:dyDescent="0.45">
@@ -7087,6 +7099,34 @@
         <v>738</v>
       </c>
       <c r="E300" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="301" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B301" t="s">
+        <v>739</v>
+      </c>
+      <c r="C301" t="s">
+        <v>740</v>
+      </c>
+      <c r="D301" t="s">
+        <v>740</v>
+      </c>
+      <c r="E301" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="302" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B302" t="s">
+        <v>741</v>
+      </c>
+      <c r="C302" t="s">
+        <v>742</v>
+      </c>
+      <c r="D302" t="s">
+        <v>742</v>
+      </c>
+      <c r="E302" t="s">
         <v>147</v>
       </c>
     </row>

</xml_diff>